<commit_message>
SPM-45 Rebuild venue unavailability on 15-minute times
The story was written before the Week 7 changes and first built on
AM / PM / Night slots. Periods are now stated as the date and time the
venue becomes unavailable and is available again, on the 15-minute grid
(Week 7 Change #1, SPM-93).

- A booking is flagged when its room-in-use time, setup and turnaround
  included, overlaps the period; meeting end to start is not an overlap.
- The coordinator's notification says alternative arrangements are
  needed (Week 7 Change #2).
- Ending a period under way rounds its end down to the grid.
- A period that is already over when saved or changed is refused.
- Test cases rewritten first (19), then the automated tests, then the
  code. Fixtures and docs follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-45_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-45_Test_Cases.xlsx
@@ -7,23 +7,26 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TC01" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TC02" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TC03" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TC04" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TC05" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TC06" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="TC07" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="TC08" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TC09" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="TC10" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="TC11" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="TC12" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="TC13" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="TC14" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="TC15" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="TC16" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="TC17" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Open Questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TC01" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TC02" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TC03" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="TC04" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TC05" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="TC06" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="TC07" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TC08" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="TC09" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="TC10" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="TC11" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="TC12" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="TC13" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="TC14" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="TC15" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="TC16" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="TC17" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="TC18" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="TC19" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -463,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -535,7 +538,7 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>A venue is marked unavailable for one whole day, with a reason</t>
+          <t>A venue is marked unavailable for part of a day, by date and time, with a reason</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -599,12 +602,12 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>A return slot earlier than the start is refused</t>
+          <t>A time that is not on the 15-minute grid is refused, and the time is named</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>AC2</t>
+          <t>AC1</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -631,7 +634,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>A return in the same slot is refused, and in the next slot is accepted</t>
+          <t>A return earlier than the start is refused</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -641,7 +644,7 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
@@ -663,17 +666,17 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Choosing Other asks for the reason, and refuses to save without it</t>
+          <t>A return at the same time as the start is refused, and 15 minutes later is accepted</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>AC6</t>
+          <t>AC2, AC1</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
@@ -695,7 +698,7 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>A period with an Other reason is saved and shows what was typed</t>
+          <t>Choosing Other asks for the reason, and refuses to save without it</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
@@ -705,7 +708,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -727,12 +730,12 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Changing a period's reason from Other to a listed one drops the typed reason</t>
+          <t>A period with an Other reason is saved and shows what was typed</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>AC5, AC6</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -759,17 +762,17 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Only the bookings in a period's slots are flagged, to the exact slot at each end</t>
+          <t>Changing a period's reason from Other to a listed one drops the typed reason</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>AC1, AC3</t>
+          <t>AC5, AC6</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
@@ -791,17 +794,17 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Widening a period flags only the bookings it newly covers</t>
+          <t>Only bookings whose times overlap the period are flagged; a booking that ends as it starts, or starts as it ends, is not</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>AC5, AC3</t>
+          <t>AC3, AC1</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
@@ -823,17 +826,17 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Shortening a period flags nothing</t>
+          <t>Widening a period by 15 minutes at each end flags only the bookings it newly overlaps</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC5, AC3</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
@@ -855,7 +858,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>A period that has not started yet can be ended, which removes it</t>
+          <t>Shortening a period flags nothing</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -865,7 +868,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -887,17 +890,17 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>A booking whose setup or turnaround slot falls in the period is flagged</t>
+          <t>A period that has not started yet can be ended, which removes it</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
@@ -919,17 +922,17 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>A pending request and a finished booking are not flagged</t>
+          <t>A booking is flagged when only its setup or turnaround time overlaps the period, and not when its setup starts as the period ends</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC3, AC5</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
@@ -951,17 +954,17 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>During its period the room stays in the catalogue, and is offered only for slots outside the period</t>
+          <t>A pending request and a finished booking are not flagged</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>AC4, AC1</t>
+          <t>AC3</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
@@ -983,17 +986,17 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>An unavailable period that is under way can be ended early</t>
+          <t>During its period the room stays in the catalogue, and is offered again from the exact time it is available</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -1015,12 +1018,12 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>A venue is available again from its return slot without anyone ending the period</t>
+          <t>An unavailable period that is under way can be ended early</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -1047,228 +1050,298 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
+          <t>A venue is available again from the stated time without anyone ending the period</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>TC18</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>SPM-45-TC18</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
           <t>Two periods that overlap can both be recorded, and the calendar identifies the overlap</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>TC19</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>SPM-45-TC19</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>A period that is already over is refused</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>AC1</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="n"/>
-    </row>
-    <row r="24" ht="71.5" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>Venue Staff can mark a venue unavailable, stating the date and slot (AM, PM or Night) it becomes unavailable and the date and slot it becomes available again.</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>SPM-45-TC01
-SPM-45-TC02
-SPM-45-TC08
-SPM-45-TC14
-SPM-45-TC17</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="31" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>The date and slot it becomes available again must be later than the date and slot it becomes unavailable.</t>
         </is>
       </c>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="9" t="n"/>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>SPM-45-TC03
-SPM-45-TC04</t>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
         </is>
       </c>
       <c r="F25" s="9" t="n"/>
     </row>
-    <row r="26" ht="58" customHeight="1">
+    <row r="26" ht="98.5" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC1</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Given a venue is unavailable for a stated period, when a booking occupies a slot within that period, then it is flagged and the Coordinator notified as for a retired venue; bookings outside the period are not flagged.</t>
+          <t>Venue Staff can mark a venue unavailable, stating the date and time it becomes unavailable and the date and time it becomes available again, on the 15-minute booking grid (see: Book Venues in 15-Minute Units, SPM-93).</t>
         </is>
       </c>
       <c r="C26" s="8" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>SPM-45-TC08
+          <t>SPM-45-TC01
+SPM-45-TC02
+SPM-45-TC03
+SPM-45-TC05
 SPM-45-TC09
-SPM-45-TC12
-SPM-45-TC13</t>
+SPM-45-TC18
+SPM-45-TC19</t>
         </is>
       </c>
       <c r="F26" s="9" t="n"/>
     </row>
-    <row r="27" ht="44.5" customHeight="1">
+    <row r="27" ht="31" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>AC2</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Given the date and slot the venue becomes available again is reached, when that slot arrives, then the venue is available again from that slot without any action by Venue Staff.</t>
+          <t>The date and time it becomes available again must be later than the date and time it becomes unavailable.</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>SPM-45-TC14
-SPM-45-TC16</t>
+          <t>SPM-45-TC04
+SPM-45-TC05</t>
         </is>
       </c>
       <c r="F27" s="9" t="n"/>
     </row>
-    <row r="28" ht="71.5" customHeight="1">
+    <row r="28" ht="58" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC3</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Venue Staff can change the dates and slots of an unavailable period, or end it early.</t>
+          <t>Given a venue is unavailable for a stated period, when a booking's occupied period (its times plus the venue's setup and turnaround) overlaps that period, then it is flagged and the Coordinator notified as for a retired venue; bookings outside the period are not flagged.</t>
         </is>
       </c>
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>SPM-45-TC07
-SPM-45-TC09
+          <t>SPM-45-TC09
 SPM-45-TC10
-SPM-45-TC11
-SPM-45-TC15</t>
+SPM-45-TC13
+SPM-45-TC14</t>
         </is>
       </c>
       <c r="F28" s="9" t="n"/>
     </row>
-    <row r="29" ht="71.5" customHeight="1">
+    <row r="29" ht="44.5" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>AC6</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Venue Staff must select the reason for an unavailable period (maintenance, equipment failure, renovation, safety, internal activity or other); when Other is selected, they must describe the reason.</t>
+          <t>Given the date and time the venue becomes available again is reached, when that time arrives, then the venue is available again from that time without any action by Venue Staff.</t>
         </is>
       </c>
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="11" t="inlineStr">
         <is>
+          <t>SPM-45-TC15
+SPM-45-TC17</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n"/>
+    </row>
+    <row r="30" ht="85" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>AC5</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Venue Staff can change the dates and times of an unavailable period, or end it early.</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>SPM-45-TC08
+SPM-45-TC10
+SPM-45-TC11
+SPM-45-TC12
+SPM-45-TC13
+SPM-45-TC16</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="71.5" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>AC6</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Venue Staff must select the reason for an unavailable period (maintenance, equipment failure, renovation, safety, internal activity or other); when Other is selected, they must describe the reason.</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
           <t>SPM-45-TC01
 SPM-45-TC02
-SPM-45-TC05
 SPM-45-TC06
-SPM-45-TC07</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="n"/>
-    </row>
-    <row r="31" ht="179.5" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
+SPM-45-TC07
+SPM-45-TC08</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n"/>
+    </row>
+    <row r="33" ht="220" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>prisma/schema.prisma
 src/lib/venueUnavailability.ts
 src/lib/venueUnavailabilityService.ts
 src/lib/venueImpact.ts
-src/lib/venueSlots.ts
+src/lib/venueTime.ts
+src/lib/venueAvailability.ts
 src/lib/validation/venues.ts
 src/app/api/venues/[id]/unavailability/route.ts
 src/app/api/venues/[id]/unavailability/[periodId]/route.ts
-src/app/api/venues/[id]/availability/route.ts
 src/components/VenueUnavailablePeriods.tsx
 src/app/venues/[id]/edit/page.tsx
 src/app/venues/[id]/availability/page.tsx
-scripts/seed-spm45.ts</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="8" t="n"/>
-      <c r="E31" s="8" t="n"/>
-      <c r="F31" s="9" t="n"/>
+src/app/venues/page.tsx
+src/lib/roles.ts
+scripts/seed-spm45.ts
+prisma/seed.ts</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E30:F30"/>
     <mergeCell ref="E29:F29"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="B31:D31"/>
     <mergeCell ref="E25:F25"/>
+    <mergeCell ref="B33:F33"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E23:F23"/>
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="E28:F28"/>
-    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B30:D30"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="E31:F31"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -1288,6 +1361,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1322,11 +1397,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC09</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="98.5" customHeight="1">
+          <t>SPM-45-TC08</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1334,13 +1409,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC08 has just been run (SPM45 Period Room is unavailable from 10 Jun 2027 PM and available again from 15 Jun 2027 PM; 'SPM45 Afternoon Workshop' and 'SPM45 Closing Seminar' are flagged).
+          <t>SPM-45-TC07 has just been run (SPM45 Dates Room has the period 25 Jul 2027, 09:00 to 26 Jul 2027, 09:00, reason Other, 'Film crew on site').
 Still logged in as Venue Staff Marcus Wong.
-Go straight on to SPM-45-TC10 and TC11, then run npm run fixtures:spm45. If you stop here, run it now.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="112" customHeight="1">
+After this case run npm run fixtures:spm45: it removes every period the Dates Room cases recorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1349,11 +1424,10 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click 'Venues' in the sidebar
-2. Click the 'SPM45 Period Room' row
-3. Click 'Change period'
-4. Change 'Unavailable from' to 9 Jun 2027 and 'First unavailable slot' to Night
-5. Change 'Available again on' to 16 Jun 2027 and 'First available slot' to AM
-6. In the dialog, click 'Save period'</t>
+2. Click the 'SPM45 Dates Room' row
+3. Click 'Change period' on the period for 25 Jul 2027
+4. In 'Reason', choose 'Internal activity'
+5. In the dialog, click 'Save period'</t>
         </is>
       </c>
     </row>
@@ -1365,13 +1439,13 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: SPM45 Period Room (SPM45-PER)
-Unavailable from: 10 Jun 2027 PM changed to 9 Jun 2027 Night
-Available again on: 15 Jun 2027 PM changed to 16 Jun 2027 AM</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="166" customHeight="1">
+          <t>Venue: SPM45 Dates Room (SPM45-DAT)
+Period: 25 Jul 2027, 09:00 to 26 Jul 2027, 09:00
+Reason: Other changed to Internal activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="152.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1379,8 +1453,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 3: A dialog titled 'Change unavailable period' appears, filled in with 10 Jun 2027, PM; 15 Jun 2027, PM and the reason 'Equipment failure'.
-Step 6: The dialog closes. An amber message titled 'Unavailable period changed — 2 bookings flagged for review, coordinators notified' lists exactly two: 'SPM45 Morning Briefing: the venue is unavailable during this booking' and 'SPM45 Return Forum: the venue is unavailable during this booking'. 'SPM45 Afternoon Workshop' and 'SPM45 Closing Seminar' are not listed again - they were already flagged. The period now reads 'Unavailable from 9 Jun 2027 Night. Available again from 16 Jun 2027 AM.'</t>
+          <t>Step 3: A dialog titled 'Change unavailable period' appears, filled in with 25 Jul 2027 and 09:00; 26 Jul 2027 and 09:00; the reason 'Other' and 'Film crew on site' in 'Other reason'.
+Step 4: The 'Other reason' field disappears.
+Step 5: The dialog closes. A green 'Unavailable period changed' message reads 'No approved bookings were affected, so nobody needed to be notified.' The period now reads 'Internal activity', 'Unavailable from 25 Jul 2027, 09:00. Available again from 26 Jul 2027, 09:00.', and 'Film crew on site' is no longer shown.</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1478,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -1489,11 +1564,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="98.5" customHeight="1">
+          <t>SPM-45-TC09</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="274" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1501,13 +1576,17 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC09 has just been run (SPM45 Period Room is unavailable from 9 Jun 2027 Night and available again from 16 Jun 2027 AM; all four bookings are flagged).
-Still logged in as Venue Staff Marcus Wong, on the 'SPM45 Period Room' page.
-Go straight on to SPM-45-TC11, then run npm run fixtures:spm45. If you stop here, run it now.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="125.5" customHeight="1">
+          <t>Fixtures: 'SPM45 Period Room' (SPM45-PER) is active, has no unavailable period and no setup or turnaround time, so a booking occupies the room for its own times only. It has four Approved bookings, none of them flagged, all with coordinator Daniel Tan:
+- 'SPM45 Morning Briefing', 10 Jun 2027, 11:00–13:00: ends as the period starts
+- 'SPM45 Afternoon Workshop', 10 Jun 2027, 13:00–15:00: starts as the period starts
+- 'SPM45 Closing Seminar', 15 Jun 2027, 10:00–13:00: ends as the period ends
+- 'SPM45 Return Forum', 15 Jun 2027, 13:00–15:00: starts as the venue is available again
+If any of it is missing, or the room already has an unavailable period because an earlier run was not reset, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+This case flags two bookings and records a period. Go straight on to SPM-45-TC10, TC11 and TC12, then run npm run fixtures:spm45. If you stop here, run it now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="179.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1515,17 +1594,21 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Change period'
-2. Change 'Unavailable from' to 12 Jun 2027 and 'First unavailable slot' to AM
-3. Change 'Available again on' to 13 Jun 2027 and 'First available slot' to AM
-4. In the dialog, click 'Save period'
-5. Click 'View availability'
-6. Set 'From' to 10 Jun 2027 and 'To' to 15 Jun 2027
-7. Click 'Show availability'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
+          <t>1. Log in as marcus.wong@connectsphere.com / password123
+2. Click 'Venues' in the sidebar
+3. Click the 'SPM45 Period Room' row
+4. Click 'Mark unavailable'
+5. Set 'Unavailable from' to 10 Jun 2027 and 'From time' to 13:00
+6. Set 'Available again on' to 15 Jun 2027 and 'Available again at' to 13:00
+7. In 'Reason', choose 'Equipment failure'
+8. In the dialog, click 'Mark unavailable'
+9. Click 'View availability'
+10. Set 'From' to 10 Jun 2027 and 'To' to 15 Jun 2027
+11. Click 'Show availability'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="71.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1533,12 +1616,14 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: SPM45 Period Room (SPM45-PER)
-Period: 9 Jun 2027 Night to 16 Jun 2027 AM, shortened to 12 Jun 2027 AM to 13 Jun 2027 AM</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="152.5" customHeight="1">
+          <t>Venue: SPM45 Period Room (SPM45-PER), setup 0 min, turnaround 0 min
+Unavailable from: 10 Jun 2027, 13:00
+Available again: 15 Jun 2027, 13:00
+Reason: Equipment failure</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="274" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1546,8 +1631,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 4: The dialog closes. A green 'Unavailable period changed' message reads 'No approved bookings were affected, so nobody needed to be notified.' - no booking is listed. The period now reads 'Unavailable from 12 Jun 2027 AM. Available again from 13 Jun 2027 AM.'
-Step 7: Only 12 Jun 2027 shows 'Unavailable' in all three slots. On 10 Jun 2027 AM and PM show 'Booked' with 'SPM45 Morning Briefing' and 'SPM45 Afternoon Workshop'; on 15 Jun 2027 AM and PM show 'Booked' with 'SPM45 Closing Seminar' and 'SPM45 Return Forum'. Every other slot from 10 to 15 Jun 2027 shows 'Free', and there is no overlap warning.</t>
+          <t>Step 8: An amber message titled 'Unavailable period saved — 2 bookings flagged for review, coordinators notified' appears. It says the bookings have not been changed, and lists exactly two: 'SPM45 Afternoon Workshop: the venue is unavailable during this booking' and 'SPM45 Closing Seminar: the venue is unavailable during this booking'. 'SPM45 Morning Briefing' and 'SPM45 Return Forum' are not listed. Under 'Unavailable periods' the period is listed: 'Equipment failure', 'Unavailable from 10 Jun 2027, 13:00. Available again from 15 Jun 2027, 13:00.'
+Step 11: The 10 Jun 2027 row lists 'Booked 11:00–13:00 · SPM45 Morning Briefing', 'Unavailable 13:00–24:00 · Equipment failure' and 'Booked 13:00–15:00 · SPM45 Afternoon Workshop'. The rows for 11, 12, 13 and 14 Jun 2027 each list 'Unavailable 00:00–24:00 · Equipment failure'. The 15 Jun 2027 row lists 'Unavailable 00:00–13:00 · Equipment failure', 'Booked 10:00–13:00 · SPM45 Closing Seminar' and 'Booked 13:00–15:00 · SPM45 Return Forum'. The warning 'Some bookings or unavailable periods overlap' is shown, because the two flagged bookings sit inside the period.</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1655,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -1656,11 +1741,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC11</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="85" customHeight="1">
+          <t>SPM-45-TC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1668,9 +1753,9 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC10 has just been run (SPM45 Period Room is unavailable from 12 Jun 2027 AM and available again from 13 Jun 2027 AM).
+          <t>SPM-45-TC09 has just been run (SPM45 Period Room is unavailable from 10 Jun 2027, 13:00 and available again from 15 Jun 2027, 13:00; 'SPM45 Afternoon Workshop' and 'SPM45 Closing Seminar' are flagged).
 Still logged in as Venue Staff Marcus Wong.
-After this case run npm run fixtures:spm45 - it removes the flags SPM-45-TC08 and TC09 put on the four bookings.</t>
+Go straight on to SPM-45-TC11 and TC12, then run npm run fixtures:spm45. If you stop here, run it now.</t>
         </is>
       </c>
     </row>
@@ -1684,14 +1769,14 @@
         <is>
           <t>1. Click 'Venues' in the sidebar
 2. Click the 'SPM45 Period Room' row
-3. Click 'End period'
-4. Click 'View availability'
-5. Set 'From' and 'To' to 12 Jun 2027
-6. Click 'Show availability'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+3. Click 'Change period'
+4. Change 'From time' to 12:45
+5. Change 'Available again at' to 13:15
+6. In the dialog, click 'Save period'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1700,11 +1785,12 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Venue: SPM45 Period Room (SPM45-PER)
-Period: 12 Jun 2027 AM to 13 Jun 2027 AM</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+Unavailable from: 10 Jun 2027, 13:00 changed to 12:45
+Available again: 15 Jun 2027, 13:00 changed to 13:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="179.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1712,8 +1798,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 3: A green 'Unavailable period ended' message appears. Under 'Unavailable periods' the text 'No unavailable periods under way or coming up.' is shown, and there is no 'Change period' or 'End period' button.
-Step 6: On 12 Jun 2027 AM, PM and Night all show 'Free', and 'Unavailable periods' reads 'No unavailable periods in this range.'</t>
+          <t>Step 3: A dialog titled 'Change unavailable period' appears, filled in with 10 Jun 2027 and 13:00; 15 Jun 2027 and 13:00; and the reason 'Equipment failure'.
+Step 6: The dialog closes. An amber message titled 'Unavailable period changed — 2 bookings flagged for review, coordinators notified' lists exactly two: 'SPM45 Morning Briefing: the venue is unavailable during this booking' (its last 15 minutes, 12:45–13:00, are now in the period) and 'SPM45 Return Forum: the venue is unavailable during this booking' (its first 15 minutes, 13:00–13:15). 'SPM45 Afternoon Workshop' and 'SPM45 Closing Seminar' are not listed again: they were already flagged. The period now reads 'Unavailable from 10 Jun 2027, 12:45. Available again from 15 Jun 2027, 13:15.'</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1822,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -1822,11 +1908,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC12</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="206.5" customHeight="1">
+          <t>SPM-45-TC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1834,16 +1920,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Setup Room' (SPM45-SET) needs a setup slot before each booking and a turnaround slot after it (60 minutes each). It has no unavailable period and three Approved bookings, none flagged, all with coordinator Daniel Tan:
-- 'SPM45 Evening Talk', 20 Jun 2027, Night - its turnaround slot is 21 Jun 2027 AM
-- 'SPM45 Afternoon Talk', 22 Jun 2027, PM - its setup slot is 22 Jun 2027 AM
-- 'SPM45 Later Talk', 23 Jun 2027, PM - its setup slot is 23 Jun 2027 AM
-If any of it is missing, or the room already has an unavailable period, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-Run npm run fixtures:spm45 after this case - it removes the period and the two flags.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="139" customHeight="1">
+          <t>SPM-45-TC10 has just been run (SPM45 Period Room is unavailable from 10 Jun 2027, 12:45 and available again from 15 Jun 2027, 13:15; all four bookings are flagged).
+Still logged in as Venue Staff Marcus Wong, on the 'SPM45 Period Room' page.
+Go straight on to SPM-45-TC12, then run npm run fixtures:spm45. If you stop here, run it now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="125.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1851,18 +1934,17 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Log in as marcus.wong@connectsphere.com / password123
-2. Click 'Venues' in the sidebar
-3. Click the 'SPM45 Setup Room' row
-4. Click 'Mark unavailable'
-5. Set 'Unavailable from' to 21 Jun 2027 and 'First unavailable slot' to AM
-6. Set 'Available again on' to 22 Jun 2027 and 'First available slot' to PM
-7. In 'Reason', choose 'Maintenance'
-8. In the dialog, click 'Mark unavailable'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
+          <t>1. Click 'Change period'
+2. Change 'Unavailable from' to 12 Jun 2027 and 'From time' to 09:00
+3. Change 'Available again on' to 12 Jun 2027 and 'Available again at' to 17:00
+4. In the dialog, click 'Save period'
+5. Click 'View availability'
+6. Set 'From' to 10 Jun 2027 and 'To' to 15 Jun 2027
+7. Click 'Show availability'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1870,14 +1952,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: SPM45 Setup Room (SPM45-SET)
-Unavailable from: 21 Jun 2027, AM
-Available again on: 22 Jun 2027, PM
-Reason: Maintenance</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="112" customHeight="1">
+          <t>Venue: SPM45 Period Room (SPM45-PER)
+Period: 10 Jun 2027, 12:45 to 15 Jun 2027, 13:15, shortened to 12 Jun 2027, 09:00 to 12 Jun 2027, 17:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="179.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1885,7 +1965,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 8: An amber message titled 'Unavailable period saved — 2 bookings flagged for review, coordinators notified' lists exactly two: 'SPM45 Evening Talk: the venue is unavailable during this booking' and 'SPM45 Afternoon Talk: the venue is unavailable during this booking'. Neither booking's own slot is in the period - the Evening Talk's turnaround slot and the Afternoon Talk's setup slot are. 'SPM45 Later Talk' is not listed.</t>
+          <t>Step 4: The dialog closes. A green 'Unavailable period changed' message reads 'No approved bookings were affected, so nobody needed to be notified.' and no booking is listed. The period now reads 'Unavailable from 12 Jun 2027, 09:00. Available again from 12 Jun 2027, 17:00.'
+Step 7: The 12 Jun 2027 row lists 'Unavailable 09:00–17:00 · Equipment failure' and nothing else. The 10 Jun 2027 row lists only 'Booked 11:00–13:00 · SPM45 Morning Briefing' and 'Booked 13:00–15:00 · SPM45 Afternoon Workshop'; the 15 Jun 2027 row lists only 'Booked 10:00–13:00 · SPM45 Closing Seminar' and 'Booked 13:00–15:00 · SPM45 Return Forum'. The rows for 11, 13 and 14 Jun 2027 show 'Free', and there is no overlap warning.</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1989,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -1994,11 +2075,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC13</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="179.5" customHeight="1">
+          <t>SPM-45-TC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2006,16 +2087,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Status Room' (SPM45-STA) has no unavailable period and three bookings, none flagged, all with coordinator Daniel Tan:
-- 'SPM45 Finished Meeting', 15 Sep 2026, AM - Approved, and already over
-- 'SPM45 Approved Review', 5 Jul 2027, AM - Approved
-- 'SPM45 Pending Request', 5 Jul 2027, PM - Pending, not yet approved
-If any of it is missing, or the room already has an unavailable period, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-Run npm run fixtures:spm45 after this case - it removes the period and the flag.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="139" customHeight="1">
+          <t>SPM-45-TC11 has just been run (SPM45 Period Room is unavailable from 12 Jun 2027, 09:00 and available again from 12 Jun 2027, 17:00).
+Still logged in as Venue Staff Marcus Wong.
+After this case run npm run fixtures:spm45: it removes the flags SPM-45-TC09 and TC10 put on the four bookings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2023,18 +2101,16 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Log in as marcus.wong@connectsphere.com / password123
-2. Click 'Venues' in the sidebar
-3. Click the 'SPM45 Status Room' row
-4. Click 'Mark unavailable'
-5. Set 'Unavailable from' to 1 Sep 2026 and 'First unavailable slot' to AM
-6. Set 'Available again on' to 7 Jul 2027 and 'First available slot' to AM
-7. In 'Reason', choose 'Renovation'
-8. In the dialog, click 'Mark unavailable'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="71.5" customHeight="1">
+          <t>1. Click 'Venues' in the sidebar
+2. Click the 'SPM45 Period Room' row
+3. Click 'End period'
+4. Click 'View availability'
+5. Set 'From' and 'To' to 12 Jun 2027
+6. Click 'Show availability'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2042,14 +2118,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: SPM45 Status Room (SPM45-STA)
-Unavailable from: 1 Sep 2026, AM
-Available again on: 7 Jul 2027, AM (covers all three bookings)
-Reason: Renovation</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
+          <t>Venue: SPM45 Period Room (SPM45-PER)
+Period: 12 Jun 2027, 09:00 to 12 Jun 2027, 17:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2057,7 +2131,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 8: An amber message titled 'Unavailable period saved — 1 booking flagged for review, coordinators notified' lists only 'SPM45 Approved Review: the venue is unavailable during this booking'. 'SPM45 Pending Request' is not listed, because a request is not yet a commitment, and 'SPM45 Finished Meeting' is not listed, because it has already taken place.</t>
+          <t>Step 3: A green 'Unavailable period ended' message appears. Under 'Unavailable periods' the text 'No unavailable periods under way or coming up.' is shown, and there is no 'Change period' or 'End period' button.
+Step 6: The 12 Jun 2027 row shows 'Free', and the 'Unavailable periods' card reads 'No unavailable periods in this range.'</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2155,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2166,11 +2241,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC14</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="125.5" customHeight="1">
+          <t>SPM-45-TC13</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="179.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2178,13 +2253,15 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Closure Room' (SPM45-NOW) has an unavailable period that is under way: Renovation, unavailable from 1 Oct 2026 AM, available again from 1 Dec 2028 AM. It is open 07:00-23:00 and has no bookings.
-If it is missing, or its period was already ended by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-This case changes nothing. Run it before SPM-45-TC15, which ends the period.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="125.5" customHeight="1">
+          <t>Fixtures: 'SPM45 Setup Room' (SPM45-SET) has a setup time of 30 minutes and a turnaround time of 45 minutes. It has no unavailable period and two Approved bookings, neither flagged, both with coordinator Daniel Tan:
+- 'SPM45 Early Talk', 21 Jun 2027, 07:30–08:30: room in use 07:00–09:15 (turnaround 08:30–09:15)
+- 'SPM45 Later Talk', 22 Jun 2027, 13:30–14:30: room in use 13:00–15:15 (setup 13:00–13:30)
+If any of it is missing, or the room already has an unavailable period, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+Run npm run fixtures:spm45 after this case: it removes the period and the two flags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="179.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2192,17 +2269,21 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Log in as daniel.tan@connectsphere.com / password123
+          <t>1. Log in as marcus.wong@connectsphere.com / password123
 2. Click 'Venues' in the sidebar
-3. Click 'Find a venue'
-4. Set 'From' to 30 Nov 2028, 19:00 and 'To' to 30 Nov 2028, 22:00
-5. Click 'Search'
-6. Change 'From' to 1 Dec 2028, 09:00 and 'To' to 1 Dec 2028, 12:00
-7. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
+3. Click the 'SPM45 Setup Room' row
+4. Click 'Mark unavailable'
+5. Set 'Unavailable from' to 21 Jun 2027 and 'From time' to 09:00
+6. Set 'Available again on' to 22 Jun 2027 and 'Available again at' to 13:00
+7. In 'Reason', choose 'Maintenance'
+8. In the dialog, click 'Mark unavailable'
+9. Click 'Change period'
+10. Change 'Available again at' to 13:15
+11. In the dialog, click 'Save period'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="71.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2210,14 +2291,14 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Account: daniel.tan@connectsphere.com (Event Coordinator)
-Venue: SPM45 Closure Room (SPM45-NOW)
-Last unavailable slot: 30 Nov 2028, Night (19:00-22:00)
-First available slot: 1 Dec 2028, AM (09:00-12:00)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
+          <t>Venue: SPM45 Setup Room (SPM45-SET), setup 30 min, turnaround 45 min
+Unavailable from: 21 Jun 2027, 09:00
+Available again: 22 Jun 2027, 13:00, then changed to 13:15
+Reason: Maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="179.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2225,9 +2306,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 2: 'SPM45 Closure Room' is in the Venues list - a room with an unavailable period is not retired.
-Step 5: 'SPM45 Closure Room' is not among the results - 30 Nov 2028 Night is the last slot of its period.
-Step 7: 'SPM45 Closure Room' is among the results - 1 Dec 2028 AM is the slot it is available again.</t>
+          <t>Step 8: An amber message titled 'Unavailable period saved — 1 booking flagged for review, coordinators notified' lists only 'SPM45 Early Talk: the venue is unavailable during this booking'. The talk itself ends at 08:30, before the period; its turnaround runs to 09:15, 15 minutes into it. 'SPM45 Later Talk' is not listed: its setup starts at 13:00, exactly when the venue is available again.
+Step 11: An amber message titled 'Unavailable period changed — 1 booking flagged for review, coordinators notified' lists only 'SPM45 Later Talk: the venue is unavailable during this booking'. The talk itself starts at 13:30, after the period; the first 15 minutes of its setup (13:00–13:15) are now in it. 'SPM45 Early Talk' is not listed again.</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2330,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2336,11 +2416,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC15</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="125.5" customHeight="1">
+          <t>SPM-45-TC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="179.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2348,13 +2428,16 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Closure Room' (SPM45-NOW) has an unavailable period that is under way: Renovation, unavailable from 1 Oct 2026 AM, available again from 1 Dec 2028 AM. It is open 07:00-23:00 and has no bookings.
-If it is missing, or its period was already ended by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-Run npm run fixtures:spm45 after this case to put the period back.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="98.5" customHeight="1">
+          <t>Fixtures: 'SPM45 Status Room' (SPM45-STA) has no unavailable period, no setup or turnaround time, and three bookings, none flagged, all with coordinator Daniel Tan:
+- 'SPM45 Finished Meeting', 15 Sep 2026, 09:00–12:00: Approved, and already over
+- 'SPM45 Approved Review', 5 Jul 2027, 09:00–12:00: Approved
+- 'SPM45 Pending Request', 5 Jul 2027, 14:00–17:00: Pending, not yet approved
+If any of it is missing, or the room already has an unavailable period, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+Run npm run fixtures:spm45 after this case: it removes the period and the flag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="139" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2364,15 +2447,16 @@
         <is>
           <t>1. Log in as marcus.wong@connectsphere.com / password123
 2. Click 'Venues' in the sidebar
-3. Click the 'SPM45 Closure Room' row
-4. Click 'End period'
-5. Click 'View availability'
-6. Set 'From' and 'To' to tomorrow's date
-7. Click 'Show availability'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
+3. Click the 'SPM45 Status Room' row
+4. Click 'Mark unavailable'
+5. Set 'Unavailable from' to 1 Sep 2026 and 'From time' to 00:00
+6. Set 'Available again on' to 7 Jul 2027 and 'Available again at' to 00:00
+7. In 'Reason', choose 'Renovation'
+8. In the dialog, click 'Mark unavailable'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="71.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2380,9 +2464,10 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: SPM45 Closure Room (SPM45-NOW)
-Period (set by the fixture script): Renovation, 1 Oct 2026 AM to 1 Dec 2028 AM
-Calendar date: tomorrow</t>
+          <t>Venue: SPM45 Status Room (SPM45-STA)
+Unavailable from: 1 Sep 2026, 00:00 (already in the past)
+Available again: 7 Jul 2027, 00:00 (the period covers all three bookings)
+Reason: Renovation</t>
         </is>
       </c>
     </row>
@@ -2394,9 +2479,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 3: Under 'Unavailable periods' one period is listed: 'Renovation', 'Unavailable from 1 Oct 2026 AM. Available again from 1 Dec 2028 AM.', with the buttons 'Change period' and 'End period'.
-Step 4: A green 'Unavailable period ended' message appears, and the period is no longer listed.
-Step 7: AM, PM and Night all show 'Free', and 'Unavailable periods' reads 'No unavailable periods in this range.' - the room did not wait for 1 Dec 2028.</t>
+          <t>Step 8: An amber message titled 'Unavailable period saved — 1 booking flagged for review, coordinators notified' lists only 'SPM45 Approved Review: the venue is unavailable during this booking'. 'SPM45 Pending Request' is not listed, because a request is not yet a commitment, and 'SPM45 Finished Meeting' is not listed, because it has already taken place. Under 'Unavailable periods' the period is listed: 'Renovation', 'Unavailable from 1 Sep 2026, 00:00. Available again from 7 Jul 2027, 00:00.'</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2502,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2505,11 +2588,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC16</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="98.5" customHeight="1">
+          <t>SPM-45-TC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="139" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2517,13 +2600,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Reopened Room' (SPM45-BAK) has an unavailable period that has passed: Maintenance, unavailable from 1 Sep 2026 AM, available again from 1 Oct 2026 AM. Nobody has ended or changed it, and the room has no bookings.
-If it is missing, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-This case changes nothing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
+          <t>Fixtures: 'SPM45 Closure Room' (SPM45-NOW) has an unavailable period that is under way: Renovation, unavailable from 1 Oct 2026, 00:00, available again from 1 Dec 2028, 09:00. It is open 07:00–23:00, has no setup or turnaround time and no bookings.
+If it is missing, or its period was already ended by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+This case changes nothing. Run it before SPM-45-TC16, which ends the period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2531,12 +2614,11 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Log in as marcus.wong@connectsphere.com / password123
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
 2. Click 'Venues' in the sidebar
-3. Click the 'SPM45 Reopened Room' row
-4. Click 'View availability'
-5. Set 'From' to 30 Sep 2026 and 'To' to 1 Oct 2026
-6. Click 'Show availability'</t>
+3. Click 'Find a venue'
+4. Set 'From' to 1 Dec 2028, 08:00 and 'To' to 1 Dec 2028, 09:00, leave every other filter empty, and click 'Search'
+5. Change 'From' to 1 Dec 2028, 09:00 and 'To' to 1 Dec 2028, 10:00 and click 'Search'</t>
         </is>
       </c>
     </row>
@@ -2548,13 +2630,14 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: SPM45 Reopened Room (SPM45-BAK)
-Period (set by the fixture script): Maintenance, 1 Sep 2026 AM to 1 Oct 2026 AM
-Calendar range: 30 Sep 2026 to 1 Oct 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="112" customHeight="1">
+          <t>Account: daniel.tan@connectsphere.com (Event Coordinator)
+Venue: SPM45 Closure Room (SPM45-NOW)
+Last hour of the period: 1 Dec 2028, 08:00–09:00
+First hour it is available: 1 Dec 2028, 09:00–10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="85" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2562,9 +2645,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 2: 'SPM45 Reopened Room' is listed with the status 'Active'.
-Step 3: Under 'Unavailable periods' the text 'No unavailable periods under way or coming up.' is shown - the period is over, so there is nothing to end.
-Step 6: On 30 Sep 2026, AM, PM and Night all show 'Unavailable'. On 1 Oct 2026, AM, PM and Night all show 'Free' - the room came back from the slot that was stated.</t>
+          <t>Step 2: 'SPM45 Closure Room' is in the Venues list: a room with an unavailable period is not retired.
+Step 4: 'SPM45 Closure Room' is not among the results: 08:00–09:00 is still inside its period.
+Step 5: 'SPM45 Closure Room' is among the results: 09:00 is the time it is available again, and nobody ended the period.</t>
         </is>
       </c>
     </row>
@@ -2587,7 +2670,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2673,11 +2756,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC17</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="98.5" customHeight="1">
+          <t>SPM-45-TC16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2685,13 +2768,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings. It has no unavailable period in August 2027.
-If it is missing, or has periods left by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-Run npm run fixtures:spm45 after this case to remove both periods.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="233.5" customHeight="1">
+          <t>Fixtures: 'SPM45 Closure Room' (SPM45-NOW) has an unavailable period that is under way: Renovation, unavailable from 1 Oct 2026, 00:00, available again from 1 Dec 2028, 09:00. It has no bookings.
+If it is missing, or its period was already ended by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+Run npm run fixtures:spm45 after this case to put the period back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2701,23 +2784,15 @@
         <is>
           <t>1. Log in as marcus.wong@connectsphere.com / password123
 2. Click 'Venues' in the sidebar
-3. Click the 'SPM45 Dates Room' row
-4. Click 'Mark unavailable'
-5. Set 'Unavailable from' to 2 Aug 2027 and 'Available again on' to 4 Aug 2027
-6. In 'Reason', choose 'Maintenance'
-7. In the dialog, click 'Mark unavailable'
-8. Click 'Mark unavailable'
-9. Set 'Unavailable from' to 3 Aug 2027 and 'First unavailable slot' to PM
-10. Set 'Available again on' to 5 Aug 2027
-11. In 'Reason', choose 'Safety'
-12. In the dialog, click 'Mark unavailable'
-13. Click 'View availability'
-14. Set 'From' to 2 Aug 2027 and 'To' to 5 Aug 2027
-15. Click 'Show availability'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
+3. Click the 'SPM45 Closure Room' row
+4. Click 'End period'
+5. Click 'View availability'
+6. Set 'From' and 'To' to tomorrow's date
+7. Click 'Show availability'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2725,13 +2800,13 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: SPM45 Dates Room (SPM45-DAT)
-First period: Maintenance, 2 Aug 2027 AM to 4 Aug 2027 AM
-Second period: Safety, 3 Aug 2027 PM to 5 Aug 2027 AM</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="166" customHeight="1">
+          <t>Venue: SPM45 Closure Room (SPM45-NOW)
+Period (set by the fixture script): Renovation, 1 Oct 2026, 00:00 to 1 Dec 2028, 09:00
+Calendar date: tomorrow</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="139" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2739,9 +2814,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 7: A green 'Unavailable period saved' message appears and the Maintenance period is listed.
-Step 12: A green 'Unavailable period saved' message appears. Both periods are listed under 'Unavailable periods', the Maintenance one first: 'Unavailable from 2 Aug 2027 AM. Available again from 4 Aug 2027 AM.' and 'Unavailable from 3 Aug 2027 PM. Available again from 5 Aug 2027 AM.'
-Step 15: Every slot from 2 Aug 2027 AM to 4 Aug 2027 Night shows 'Unavailable', and 5 Aug 2027 shows 'Free' in all three slots. The warning 'Some bookings or unavailable periods overlap' is shown, and under 'Unavailable periods' the Maintenance and Safety periods each carry an 'Overlaps with' note.</t>
+          <t>Step 3: Under 'Unavailable periods' one period is listed: 'Renovation', 'Unavailable from 1 Oct 2026, 00:00. Available again from 1 Dec 2028, 09:00.', with the buttons 'Change period' and 'End period'.
+Step 4: A green 'Unavailable period ended' message appears, and the period is no longer listed: the text 'No unavailable periods under way or coming up.' is shown.
+Step 7: Tomorrow's row shows 'Free', and the 'Unavailable periods' card reads 'No unavailable periods in this range.': the room did not wait for 1 Dec 2028.</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2839,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2821,7 +2896,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2850,11 +2925,303 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC01</t>
-        </is>
-      </c>
+          <t>SPM-45-TC17</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="98.5" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Fixtures: 'SPM45 Reopened Room' (SPM45-BAK) has an unavailable period that has passed: Maintenance, unavailable from 1 Sep 2026, 00:00, available again from 1 Oct 2026, 12:00. Nobody has ended or changed it, and the room has no bookings.
+If it is missing, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+This case changes nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>1. Log in as marcus.wong@connectsphere.com / password123
+2. Click 'Venues' in the sidebar
+3. Click the 'SPM45 Reopened Room' row
+4. Click 'View availability'
+5. Set 'From' to 30 Sep 2026 and 'To' to 1 Oct 2026
+6. Click 'Show availability'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Venue: SPM45 Reopened Room (SPM45-BAK)
+Period (set by the fixture script): Maintenance, 1 Sep 2026, 00:00 to 1 Oct 2026, 12:00
+Calendar range: 30 Sep 2026 to 1 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="125.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Step 2: 'SPM45 Reopened Room' is listed with the status 'Active'.
+Step 3: Under 'Unavailable periods' the text 'No unavailable periods under way or coming up.' is shown: the period is over, so there is nothing to end.
+Step 6: The 30 Sep 2026 row lists 'Unavailable 00:00–24:00 · Maintenance'. The 1 Oct 2026 row lists 'Unavailable 00:00–12:00 · Maintenance' and nothing after 12:00: the room came back at the time that was stated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>kayalvizhi24</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Question / ambiguity for the PO or developer</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="152.5" customHeight="1">
+      <c r="A2" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Rewritten on 2026-10-09, before the code was reworked (test cases first). The 17 cases of 2026-10-06 were written for AM / PM / Night slots. SPM-45 was drafted before the Week 7 Customer Changes; Change #1 and the customer's answers #126 and #128 then replaced the slots with times on a 15-minute grid (SPM-93, Done), and SPM-45's acceptance criteria were reworded in Jira to match, so every case is new. The automated tests were rewritten next and the code then reworked to them (2026-10-09): every label and message quoted in the cases is what the code now shows. The cases have not been run by hand yet. Entries marked DECIDED were chosen here rather than taken from the story; change them in code and cases together.</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="n"/>
     </row>
     <row r="3" ht="112" customHeight="1">
+      <c r="A3" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-09 (AC1): the 'Mark &lt;venue&gt; unavailable' dialog replaces the two slot pickers with time fields. Fields: 'Unavailable from' (date), 'From time' (time), 'Available again on' (date), 'Available again at' (time), 'Reason' (picker, required), 'Other reason' (text, shown and required only when the reason is Other; 500 characters at most). All four date and time fields open empty and are required. The time fields accept any minute, as on the booking request page (SPM-93), so an off-grid time reaches the page's own message.</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n"/>
+    </row>
+    <row r="4" ht="139" customHeight="1">
+      <c r="A4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-09: messages, each shown under its field. 'Enter the date the venue becomes unavailable.', 'Enter the time the venue becomes unavailable.', 'Enter the date the venue becomes available again.', 'Enter the time the venue becomes available again.', 'Choose a time on a 15-minute step (:00, :15, :30 or :45).' (under whichever time is off the grid; the wording follows SPM-93's), 'The venue must become available again after it becomes unavailable.' (under 'Available again at'), 'This period is already over.' (under 'Available again at'), 'Choose a reason.', 'Describe the reason.' The server applies the same checks.</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n"/>
+    </row>
+    <row r="5" ht="98.5" customHeight="1">
+      <c r="A5" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-09: a period is stored exactly as stated, from the time the venue becomes unavailable to the time it is available again, Singapore time (#36). The shortest period is one 15-minute step (TC05). A period is not limited to the venue's opening hours: 00:00 is accepted (TC14), since a renovation does not stop when the room closes. The latest time that can be typed is 23:45; a period running to midnight is stated as 00:00 the next day.</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n"/>
+    </row>
+    <row r="6" ht="179.5" customHeight="1">
+      <c r="A6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-09: on the venue page each period under way or still to come is listed as its reason, the typed reason when it is Other, and 'Unavailable from &lt;date&gt;, &lt;time&gt;. Available again from &lt;date&gt;, &lt;time&gt;.' (e.g. 'Unavailable from 10 Jun 2027, 13:00. Available again from 15 Jun 2027, 13:00.'), with 'Change period' and 'End period'. Periods that are over are not listed. Kept from the earlier build: the section title 'Unavailable periods', 'No unavailable periods under way or coming up.', the message titles 'Unavailable period saved', 'Unavailable period changed' and 'Unavailable period ended', the dialog 'Change unavailable period' with 'Save period', and the flag wording 'the venue is unavailable during this booking'. Wording that says 'slots' becomes 'times' (the section's description, the dialog's first sentence, and the 'ended' message).</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n"/>
+    </row>
+    <row r="7" ht="112" customHeight="1">
+      <c r="A7" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-09 (AC3): a booking is flagged when its room-in-use period, from its start minus the venue's setup time to its end plus the venue's turnaround time, overlaps the unavailable period. This is the rule SPM-93 uses everywhere (AC6, AC7): periods that only meet end to start do not overlap, so a booking that ends as the period starts, or whose setup starts as the venue is available again, is not flagged (TC09, TC13). Only Approved bookings that have not finished are flagged (TC14), as when a venue is retired (SPM-39).</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n"/>
+    </row>
+    <row r="8" ht="139" customHeight="1">
+      <c r="A8" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-10-09 (AC5): 'End period' on a period that has not started removes it (TC12). On a period under way it brings the return time forward to the current time, rounded down to the 15-minute grid, so the room is free straight away and the stored time stays on the grid; the calendar keeps showing the time it really was unavailable. TC16 checks tomorrow rather than today for that reason. There is no confirmation dialog: ending loses nothing, and a period can be marked again. Widening a period flags the bookings it newly overlaps and does not flag an already-flagged booking again (TC10, TC13); shortening one flags nothing (TC11).</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n"/>
+    </row>
+    <row r="9" ht="233.5" customHeight="1">
+      <c r="A9" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Fixtures: scripts/seed-spm45.ts (npm run fixtures:spm45) and its copy at the end of prisma/seed.ts were reworked to times on 2026-10-09. No schema change. Rooms, all open 07:00–23:00: 'SPM45 Dates Room' (SPM45-DAT; setup 0, turnaround 0; no bookings, no period); 'SPM45 Period Room' (SPM45-PER; 0 and 0; four Approved bookings on 10 and 15 Jun 2027); 'SPM45 Setup Room' (SPM45-SET; setup 30, turnaround 45; two Approved bookings on 21 and 22 Jun 2027); 'SPM45 Status Room' (SPM45-STA; 0 and 0; an Approved, a Pending and a finished booking); 'SPM45 Closure Room' (SPM45-NOW; period Renovation, 1 Oct 2026 00:00 to 1 Dec 2028 09:00); 'SPM45 Reopened Room' (SPM45-BAK; period Maintenance, 1 Sep 2026 00:00 to 1 Oct 2026 12:00). Nine events (seed keys spm45_…), coordinator Daniel Tan, each event's own times the same as its booking's. Every run resets the rooms' periods and the events' bookings and notifications in place, and removes the one fixture event the slot-based set had that this one does not ('SPM45 Later Talk' of 23 Jun 2027). The script must be run once against the shared database before the cases can be run.</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-45-TC18</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2862,13 +3229,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings. It has no unavailable period on 9 to 11 Jun 2027.
+          <t>Fixtures: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings. It has no unavailable period in August 2027.
 If it is missing, or has periods left by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-This case records a period. The Dates Room cases (SPM-45-TC01 to TC07) can be run one after another without a reset; run npm run fixtures:spm45 after the last one you run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="179.5" customHeight="1">
+Run npm run fixtures:spm45 after this case to remove both periods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="274" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2880,17 +3247,22 @@
 2. Click 'Venues' in the sidebar
 3. Click the 'SPM45 Dates Room' row
 4. Click 'Mark unavailable'
-5. Set 'Unavailable from' to 10 Jun 2027 and 'First unavailable slot' to AM
-6. Set 'Available again on' to 11 Jun 2027 and 'First available slot' to AM
+5. Set 'Unavailable from' to 2 Aug 2027 and 'From time' to 09:00
+6. Set 'Available again on' to 4 Aug 2027 and 'Available again at' to 09:00
 7. In 'Reason', choose 'Maintenance'
 8. In the dialog, click 'Mark unavailable'
-9. Click 'View availability'
-10. Set 'From' to 9 Jun 2027 and 'To' to 11 Jun 2027
-11. Click 'Show availability'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
+9. Click 'Mark unavailable'
+10. Set 'Unavailable from' to 3 Aug 2027 and 'From time' to 14:00
+11. Set 'Available again on' to 5 Aug 2027 and 'Available again at' to 09:00
+12. In 'Reason', choose 'Safety'
+13. In the dialog, click 'Mark unavailable'
+14. Click 'View availability'
+15. Set 'From' to 2 Aug 2027 and 'To' to 5 Aug 2027
+16. Click 'Show availability'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="71.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2899,13 +3271,12 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Venue: SPM45 Dates Room (SPM45-DAT)
-Unavailable from: 10 Jun 2027, AM
-Available again on: 11 Jun 2027, AM
-Reason: Maintenance</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="301" customHeight="1">
+First period: Maintenance, 2 Aug 2027, 09:00 to 4 Aug 2027, 09:00
+Second period: Safety, 3 Aug 2027, 14:00 to 5 Aug 2027, 09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="220" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2913,10 +3284,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 3: The page has an 'Unavailable periods' section with a 'Mark unavailable' button.
-Step 4: A dialog titled 'Mark SPM45 Dates Room unavailable' appears. It has the empty date fields 'Unavailable from' and 'Available again on', the pickers 'First unavailable slot' and 'First available slot' (each offering AM, PM and Night), and a 'Reason' picker showing 'Choose a reason' and offering Maintenance, Equipment failure, Renovation, Safety, Internal activity and Other. It says that no booking is cancelled or moved.
-Step 8: The dialog closes. A green 'Unavailable period saved' message reads 'No approved bookings were affected, so nobody needed to be notified.' Under 'Unavailable periods' a period is listed: 'Maintenance', 'Unavailable from 10 Jun 2027 AM. Available again from 11 Jun 2027 AM.', with the buttons 'Change period' and 'End period'. There is no 'Retired' label beside the venue's name.
-Step 11: On 9 Jun 2027 all three slots show 'Free'. On 10 Jun 2027 AM, PM and Night all show 'Unavailable'. On 11 Jun 2027 all three slots show 'Free'. Under 'Unavailable periods' the period is listed as 'Maintenance', 10 Jun 2027 to 11 Jun 2027.</t>
+          <t>Step 8: A green 'Unavailable period saved' message appears and the Maintenance period is listed.
+Step 13: A green 'Unavailable period saved' message appears. Both periods are listed under 'Unavailable periods', the Maintenance one first: 'Unavailable from 2 Aug 2027, 09:00. Available again from 4 Aug 2027, 09:00.' and 'Unavailable from 3 Aug 2027, 14:00. Available again from 5 Aug 2027, 09:00.'
+Step 16: The 2 Aug 2027 row lists 'Unavailable 09:00–24:00 · Maintenance'. The 3 Aug 2027 row lists 'Unavailable 00:00–24:00 · Maintenance' and 'Unavailable 14:00–24:00 · Safety'. The 4 Aug 2027 row lists 'Unavailable 00:00–09:00 · Maintenance' and 'Unavailable 00:00–24:00 · Safety'. The 5 Aug 2027 row lists 'Unavailable 00:00–09:00 · Safety'. The warning 'Some bookings or unavailable periods overlap' is shown, and in the 'Unavailable periods' card the Maintenance and Safety periods each carry an 'Overlaps with' note.</t>
         </is>
       </c>
     </row>
@@ -2939,7 +3309,178 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-45-TC19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="71.5" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Fixtures: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings.
+If it is missing, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+This case changes nothing: the save is refused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="152.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>1. Log in as marcus.wong@connectsphere.com / password123
+2. Click 'Venues' in the sidebar
+3. Click the 'SPM45 Dates Room' row
+4. Click 'Mark unavailable'
+5. Set 'Unavailable from' to 1 Sep 2026 and 'From time' to 09:00
+6. Set 'Available again on' to 5 Sep 2026 and 'Available again at' to 17:00
+7. In 'Reason', choose 'Maintenance'
+8. In the dialog, click 'Mark unavailable'
+9. In the dialog, click 'Cancel'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="71.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Venue: SPM45 Dates Room (SPM45-DAT)
+Unavailable from: 1 Sep 2026, 09:00
+Available again: 5 Sep 2026, 17:00 (later than the start, but already in the past)
+Reason: Maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Step 8: The dialog stays open. Under 'Available again at' the message 'This period is already over.' appears. No 'Unavailable period saved' message appears.
+Step 9: The dialog closes. Under 'Unavailable periods' no period for September 2026 has been added.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>kayalvizhi24</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3025,11 +3566,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="85" customHeight="1">
+          <t>SPM-45-TC01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3037,13 +3578,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings. 
+          <t>Fixtures: 'SPM45 Dates Room' (SPM45-DAT) is active, has no setup or turnaround time, no bookings and no unavailable period.
 If it is missing, or has periods left by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-This case changes nothing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
+This case records a period. The Dates Room cases (SPM-45-TC01 to TC08) can be run one after another without a reset; run npm run fixtures:spm45 after the last one you run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="179.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3055,12 +3596,17 @@
 2. Click 'Venues' in the sidebar
 3. Click the 'SPM45 Dates Room' row
 4. Click 'Mark unavailable'
-5. In the dialog, click 'Mark unavailable'
-6. In the dialog, click 'Cancel'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+5. Set 'Unavailable from' to 10 Jun 2027 and 'From time' to 09:00
+6. Set 'Available again on' to 10 Jun 2027 and 'Available again at' to 17:30
+7. In 'Reason', choose 'Maintenance'
+8. In the dialog, click 'Mark unavailable'
+9. Click 'View availability'
+10. Set 'From' to 9 Jun 2027 and 'To' to 11 Jun 2027
+11. Click 'Show availability'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -3069,11 +3615,13 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Venue: SPM45 Dates Room (SPM45-DAT)
-All fields left as the dialog opens</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="112" customHeight="1">
+Unavailable from: 10 Jun 2027, 09:00
+Available again: 10 Jun 2027, 17:30
+Reason: Maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="314.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3081,8 +3629,10 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 5: The dialog stays open. Under 'Unavailable from' the message 'Enter the date the venue becomes unavailable.' appears, under 'Available again on' the message 'Enter the date the venue becomes available again.', and under 'Reason' the message 'Choose a reason.'
-Step 6: The dialog closes. No 'Unavailable period saved' message appears, and no period has been added under 'Unavailable periods'.</t>
+          <t>Step 3: The page has an 'Unavailable periods' section with a 'Mark unavailable' button and the text 'No unavailable periods under way or coming up.'
+Step 4: A dialog titled 'Mark SPM45 Dates Room unavailable' appears. It has the empty date fields 'Unavailable from' and 'Available again on', the empty time fields 'From time' and 'Available again at', and a 'Reason' picker showing 'Choose a reason' and offering Maintenance, Equipment failure, Renovation, Safety, Internal activity and Other. There are no AM, PM or Night options. It says that no booking is cancelled or moved.
+Step 8: The dialog closes. A green 'Unavailable period saved' message reads 'No approved bookings were affected, so nobody needed to be notified.' Under 'Unavailable periods' a period is listed: 'Maintenance', 'Unavailable from 10 Jun 2027, 09:00. Available again from 10 Jun 2027, 17:30.', with the buttons 'Change period' and 'End period'. There is no 'Retired' label beside the venue's name.
+Step 11: The 9 Jun 2027 row shows 'Free'. The 10 Jun 2027 row lists 'Unavailable 09:00–17:30 · Maintenance' and nothing else. The 11 Jun 2027 row shows 'Free'. The 'Unavailable periods' card lists 'Maintenance' with '10 Jun 2027, 09:00–17:30'.</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3655,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3191,11 +3741,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC03</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="85" customHeight="1">
+          <t>SPM-45-TC02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3203,13 +3753,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings. 
-If it is missing, or has periods left by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+          <t>Fixtures: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings.
+If it is missing, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
 This case changes nothing.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="193" customHeight="1">
+    <row r="4" ht="85" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3221,17 +3771,12 @@
 2. Click 'Venues' in the sidebar
 3. Click the 'SPM45 Dates Room' row
 4. Click 'Mark unavailable'
-5. Set 'Unavailable from' to 20 Jul 2027 and 'First unavailable slot' to PM
-6. Set 'Available again on' to 20 Jul 2027 and 'First available slot' to AM
-7. In 'Reason', choose 'Safety'
-8. In the dialog, click 'Mark unavailable'
-9. Change 'Available again on' to 19 Jul 2027 and 'First available slot' to Night
-10. In the dialog, click 'Mark unavailable'
-11. In the dialog, click 'Cancel'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="71.5" customHeight="1">
+5. In the dialog, click 'Mark unavailable'
+6. In the dialog, click 'Cancel'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -3240,13 +3785,11 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Venue: SPM45 Dates Room (SPM45-DAT)
-Unavailable from: 20 Jul 2027, PM
-Available again on: 20 Jul 2027, AM (earlier slot, same day), then 19 Jul 2027, Night (earlier day)
-Reason: Safety</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
+All fields left as the dialog opens</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="152.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3254,9 +3797,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 8: The dialog stays open. Under 'Available again on' the message 'The venue must become available again after it becomes unavailable.' appears.
-Step 10: The dialog stays open with the same message.
-Step 11: The dialog closes. No period for 20 Jul 2027 has been added under 'Unavailable periods'.</t>
+          <t>Step 5: The dialog stays open. Under 'Unavailable from' the message 'Enter the date the venue becomes unavailable.' appears, under 'From time' the message 'Enter the time the venue becomes unavailable.', under 'Available again on' the message 'Enter the date the venue becomes available again.', under 'Available again at' the message 'Enter the time the venue becomes available again.', and under 'Reason' the message 'Choose a reason.'
+Step 6: The dialog closes. No 'Unavailable period saved' message appears, and no period has been added under 'Unavailable periods'.</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3821,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3365,11 +3907,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC04</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="98.5" customHeight="1">
+          <t>SPM-45-TC03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3377,13 +3919,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings. It has no unavailable period on 20 Jul 2027.
-If it is missing, or has periods left by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-This case records a one-slot period. Run npm run fixtures:spm45 after the last Dates Room case you run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="206.5" customHeight="1">
+          <t>Fixtures: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings.
+If it is missing, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+This case changes nothing: every save is refused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="193" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3395,15 +3937,13 @@
 2. Click 'Venues' in the sidebar
 3. Click the 'SPM45 Dates Room' row
 4. Click 'Mark unavailable'
-5. Set 'Unavailable from' to 20 Jul 2027 and 'First unavailable slot' to PM
-6. Set 'Available again on' to 20 Jul 2027 and 'First available slot' to PM
+5. Set 'Unavailable from' to 20 Jul 2027 and 'From time' to 09:10
+6. Set 'Available again on' to 20 Jul 2027 and 'Available again at' to 17:00
 7. In 'Reason', choose 'Safety'
 8. In the dialog, click 'Mark unavailable'
-9. Change 'First available slot' to Night
+9. Change 'From time' to 09:15 and 'Available again at' to 17:40
 10. In the dialog, click 'Mark unavailable'
-11. Click 'View availability'
-12. Set 'From' and 'To' to 20 Jul 2027
-13. Click 'Show availability'</t>
+11. In the dialog, click 'Cancel'</t>
         </is>
       </c>
     </row>
@@ -3416,13 +3956,13 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Venue: SPM45 Dates Room (SPM45-DAT)
-Unavailable from: 20 Jul 2027, PM
-Available again on: 20 Jul 2027 - PM (same slot, refused), then Night (next slot, accepted)
+Date: 20 Jul 2027 for both
+Times tried: from 09:10 (off the grid) to 17:00; then from 09:15 to 17:40 (off the grid)
 Reason: Safety</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="139" customHeight="1">
+    <row r="6" ht="125.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3430,9 +3970,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 8: The dialog stays open. Under 'Available again on' the message 'The venue must become available again after it becomes unavailable.' appears - a period of no slots is refused.
-Step 10: The dialog closes. A green 'Unavailable period saved' message appears. Under 'Unavailable periods' a period is listed: 'Safety', 'Unavailable from 20 Jul 2027 PM. Available again from 20 Jul 2027 Night.'
-Step 13: On 20 Jul 2027 AM shows 'Free', PM shows 'Unavailable' and Night shows 'Free' - a period of exactly one slot.</t>
+          <t>Step 8: The dialog stays open. Under 'From time' the message 'Choose a time on a 15-minute step (:00, :15, :30 or :45).' appears. 'Available again at' has no message.
+Step 10: The dialog stays open. The message under 'From time' is gone, and under 'Available again at' the message 'Choose a time on a 15-minute step (:00, :15, :30 or :45).' appears.
+Step 11: The dialog closes. No period for 20 Jul 2027 has been added under 'Unavailable periods'.</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3995,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3541,11 +4081,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC05</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="85" customHeight="1">
+          <t>SPM-45-TC04</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3553,13 +4093,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings. 
-If it is missing, or has periods left by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-This case changes nothing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="166" customHeight="1">
+          <t>Fixtures: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings.
+If it is missing, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+This case changes nothing: every save is refused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="193" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3571,11 +4111,11 @@
 2. Click 'Venues' in the sidebar
 3. Click the 'SPM45 Dates Room' row
 4. Click 'Mark unavailable'
-5. Set 'Unavailable from' to 25 Jul 2027 and 'Available again on' to 26 Jul 2027
-6. In 'Reason', choose 'Renovation'
-7. In 'Reason', choose 'Other'
+5. Set 'Unavailable from' to 20 Jul 2027 and 'From time' to 14:00
+6. Set 'Available again on' to 20 Jul 2027 and 'Available again at' to 09:00
+7. In 'Reason', choose 'Safety'
 8. In the dialog, click 'Mark unavailable'
-9. Type three spaces into 'Other reason'
+9. Change 'Available again on' to 19 Jul 2027 and 'Available again at' to 23:45
 10. In the dialog, click 'Mark unavailable'
 11. In the dialog, click 'Cancel'</t>
         </is>
@@ -3590,14 +4130,13 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Venue: SPM45 Dates Room (SPM45-DAT)
-Unavailable from: 25 Jul 2027, AM
-Available again on: 26 Jul 2027, AM
-Reason: Renovation, then Other
-Other reason: left empty, then three spaces</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="139" customHeight="1">
+Unavailable from: 20 Jul 2027, 14:00
+Available again: 20 Jul 2027, 09:00 (earlier time, same day), then 19 Jul 2027, 23:45 (earlier day, later time of day)
+Reason: Safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3605,11 +4144,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 6: No 'Other reason' field is shown - it is only asked for when the reason is Other.
-Step 7: An empty text field 'Other reason' appears under 'Reason'.
-Step 8: The dialog stays open. Under 'Other reason' the message 'Describe the reason.' appears.
-Step 10: The dialog stays open with the same message - spaces alone are not a reason.
-Step 11: The dialog closes. No period for 25 Jul 2027 has been added under 'Unavailable periods'.</t>
+          <t>Step 8: The dialog stays open. Under 'Available again at' the message 'The venue must become available again after it becomes unavailable.' appears.
+Step 10: The dialog stays open with the same message: the date is earlier, even though 23:45 is later in the day than 14:00.
+Step 11: The dialog closes. No period for 20 Jul 2027 has been added under 'Unavailable periods'.</t>
         </is>
       </c>
     </row>
@@ -3632,7 +4169,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3718,11 +4255,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC06</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="112" customHeight="1">
+          <t>SPM-45-TC05</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3730,13 +4267,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings. It has no unavailable period on 25 Jul 2027.
+          <t>Fixtures: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings. It has no unavailable period on 20 Jul 2027.
 If it is missing, or has periods left by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-This case records a period. Go straight on to SPM-45-TC07; run npm run fixtures:spm45 after the last Dates Room case you run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="166" customHeight="1">
+This case records a 15-minute period. Run npm run fixtures:spm45 after the last Dates Room case you run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="206.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3748,13 +4285,15 @@
 2. Click 'Venues' in the sidebar
 3. Click the 'SPM45 Dates Room' row
 4. Click 'Mark unavailable'
-5. Set 'Unavailable from' to 25 Jul 2027 and 'Available again on' to 26 Jul 2027
-6. In 'Reason', choose 'Other'
-7. Type the reason into 'Other reason'
+5. Set 'Unavailable from' to 20 Jul 2027 and 'From time' to 14:00
+6. Set 'Available again on' to 20 Jul 2027 and 'Available again at' to 14:00
+7. In 'Reason', choose 'Safety'
 8. In the dialog, click 'Mark unavailable'
-9. Click 'View availability'
-10. Set 'From' and 'To' to 25 Jul 2027
-11. Click 'Show availability'</t>
+9. Change 'Available again at' to 14:15
+10. In the dialog, click 'Mark unavailable'
+11. Click 'View availability'
+12. Set 'From' and 'To' to 20 Jul 2027
+13. Click 'Show availability'</t>
         </is>
       </c>
     </row>
@@ -3767,14 +4306,13 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Venue: SPM45 Dates Room (SPM45-DAT)
-Unavailable from: 25 Jul 2027, AM
-Available again on: 26 Jul 2027, AM
-Reason: Other
-Other reason: Film crew on site</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+Unavailable from: 20 Jul 2027, 14:00
+Available again: 20 Jul 2027, 14:00 (same time, refused), then 14:15 (one 15-minute step later, accepted)
+Reason: Safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="139" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3782,8 +4320,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 8: The dialog closes. A green 'Unavailable period saved' message appears. Under 'Unavailable periods' a period is listed: 'Other', 'Film crew on site', 'Unavailable from 25 Jul 2027 AM. Available again from 26 Jul 2027 AM.'
-Step 11: On 25 Jul 2027 all three slots show 'Unavailable'. Under 'Unavailable periods' the period is listed as 'Other', 'Film crew on site', 25 Jul 2027 to 26 Jul 2027.</t>
+          <t>Step 8: The dialog stays open. Under 'Available again at' the message 'The venue must become available again after it becomes unavailable.' appears: a period of no time is refused.
+Step 10: The dialog closes. A green 'Unavailable period saved' message appears. Under 'Unavailable periods' a period is listed: 'Safety', 'Unavailable from 20 Jul 2027, 14:00. Available again from 20 Jul 2027, 14:15.'
+Step 13: The 20 Jul 2027 row lists 'Unavailable 14:00–14:15 · Safety' and nothing else: the shortest period, one 15-minute step.</t>
         </is>
       </c>
     </row>
@@ -3806,7 +4345,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3892,11 +4431,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC07</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="85" customHeight="1">
+          <t>SPM-45-TC06</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3904,13 +4443,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC06 has just been run (SPM45 Dates Room has the period 25 Jul 2027 AM to 26 Jul 2027 AM, reason Other, 'Film crew on site').
-Still logged in as Venue Staff Marcus Wong.
-After this case run npm run fixtures:spm45 - it removes every period the Dates Room cases recorded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.5" customHeight="1">
+          <t>Fixtures: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings.
+If it is missing, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+This case changes nothing: every save is refused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="193" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3918,15 +4457,22 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Venues' in the sidebar
-2. Click the 'SPM45 Dates Room' row
-3. Click 'Change period' on the period for 25 Jul 2027
-4. In 'Reason', choose 'Internal activity'
-5. In the dialog, click 'Save period'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
+          <t>1. Log in as marcus.wong@connectsphere.com / password123
+2. Click 'Venues' in the sidebar
+3. Click the 'SPM45 Dates Room' row
+4. Click 'Mark unavailable'
+5. Set 'Unavailable from' to 25 Jul 2027 and 'From time' to 09:00
+6. Set 'Available again on' to 26 Jul 2027 and 'Available again at' to 09:00
+7. In 'Reason', choose 'Renovation'
+8. In 'Reason', choose 'Other'
+9. In the dialog, click 'Mark unavailable'
+10. Type three spaces into 'Other reason'
+11. In the dialog, click 'Mark unavailable'
+12. In the dialog, click 'Cancel'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="71.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -3935,8 +4481,10 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Venue: SPM45 Dates Room (SPM45-DAT)
-Period: 25 Jul 2027 AM to 26 Jul 2027 AM
-Reason: Other changed to Internal activity</t>
+Unavailable from: 25 Jul 2027, 09:00
+Available again: 26 Jul 2027, 09:00
+Reason: Renovation, then Other
+Other reason: left empty, then three spaces</t>
         </is>
       </c>
     </row>
@@ -3948,9 +4496,11 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 3: A dialog titled 'Change unavailable period' appears, filled in with 25 Jul 2027, AM; 26 Jul 2027, AM; the reason 'Other' and 'Film crew on site' in 'Other reason'.
-Step 4: The 'Other reason' field disappears.
-Step 5: The dialog closes. A green 'Unavailable period changed' message reads 'No approved bookings were affected, so nobody needed to be notified.' The period now reads 'Internal activity', 'Unavailable from 25 Jul 2027 AM. Available again from 26 Jul 2027 AM.', and 'Film crew on site' is no longer shown.</t>
+          <t>Step 7: No 'Other reason' field is shown: it is only asked for when the reason is Other.
+Step 8: An empty text field 'Other reason' appears under 'Reason'.
+Step 9: The dialog stays open. Under 'Other reason' the message 'Describe the reason.' appears.
+Step 11: The dialog stays open with the same message: spaces alone are not a reason.
+Step 12: The dialog closes. No period for 25 Jul 2027 has been added under 'Unavailable periods'.</t>
         </is>
       </c>
     </row>
@@ -3973,7 +4523,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -4059,11 +4609,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-45-TC08</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="260.5" customHeight="1">
+          <t>SPM-45-TC07</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4071,17 +4621,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed: 'SPM45 Period Room' (SPM45-PER) is active, has no unavailable period and no setup or turnaround time. It has four Approved bookings, none of them flagged, all with coordinator Daniel Tan:
-- 'SPM45 Morning Briefing', 10 Jun 2027, AM - the slot before the period starts
-- 'SPM45 Afternoon Workshop', 10 Jun 2027, PM - the first slot of the period
-- 'SPM45 Closing Seminar', 15 Jun 2027, AM - the last slot of the period
-- 'SPM45 Return Forum', 15 Jun 2027, PM - the slot the venue is available again
-If any of it is missing, or the room already has an unavailable period because an earlier run was not reset, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
-This case flags two bookings and records a period. Go straight on to SPM-45-TC09, TC10 and TC11, then run npm run fixtures:spm45. If you stop here, run it now.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="179.5" customHeight="1">
+          <t>Fixtures: 'SPM45 Dates Room' (SPM45-DAT) is active and has no bookings. It has no unavailable period on 25 Jul 2027.
+If it is missing, or has periods left by an earlier run, run: npm run fixtures:spm45 (adds or resets the SPM45 test data without a reseed).
+This case records a period. Go straight on to SPM-45-TC08; run npm run fixtures:spm45 after the last Dates Room case you run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="193" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -4091,19 +4637,20 @@
         <is>
           <t>1. Log in as marcus.wong@connectsphere.com / password123
 2. Click 'Venues' in the sidebar
-3. Click the 'SPM45 Period Room' row
+3. Click the 'SPM45 Dates Room' row
 4. Click 'Mark unavailable'
-5. Set 'Unavailable from' to 10 Jun 2027 and 'First unavailable slot' to PM
-6. Set 'Available again on' to 15 Jun 2027 and 'First available slot' to PM
-7. In 'Reason', choose 'Equipment failure'
-8. In the dialog, click 'Mark unavailable'
-9. Click 'View availability'
-10. Set 'From' to 10 Jun 2027 and 'To' to 15 Jun 2027
-11. Click 'Show availability'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
+5. Set 'Unavailable from' to 25 Jul 2027 and 'From time' to 09:00
+6. Set 'Available again on' to 26 Jul 2027 and 'Available again at' to 09:00
+7. In 'Reason', choose 'Other'
+8. Type the reason into 'Other reason'
+9. In the dialog, click 'Mark unavailable'
+10. Click 'View availability'
+11. Set 'From' and 'To' to 25 Jul 2027
+12. Click 'Show availability'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="71.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -4111,14 +4658,15 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: SPM45 Period Room (SPM45-PER)
-Unavailable from: 10 Jun 2027, PM
-Available again on: 15 Jun 2027, PM
-Reason: Equipment failure</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="233.5" customHeight="1">
+          <t>Venue: SPM45 Dates Room (SPM45-DAT)
+Unavailable from: 25 Jul 2027, 09:00
+Available again: 26 Jul 2027, 09:00
+Reason: Other
+Other reason: Film crew on site</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -4126,8 +4674,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 8: An amber message titled 'Unavailable period saved — 2 bookings flagged for review, coordinators notified' appears. It says the bookings have not been changed, and lists exactly two: 'SPM45 Afternoon Workshop: the venue is unavailable during this booking' and 'SPM45 Closing Seminar: the venue is unavailable during this booking'. 'SPM45 Morning Briefing' and 'SPM45 Return Forum' are not listed. Under 'Unavailable periods' the period is listed: 'Equipment failure', 'Unavailable from 10 Jun 2027 PM. Available again from 15 Jun 2027 PM.'
-Step 11: On 10 Jun 2027, AM shows 'Booked' with 'SPM45 Morning Briefing', and PM and Night show 'Unavailable'. On 11 to 14 Jun 2027 every slot shows 'Unavailable'. On 15 Jun 2027, AM shows 'Unavailable', PM shows 'Booked' with 'SPM45 Return Forum', and Night shows 'Free'. The warning 'Some bookings or unavailable periods overlap' is shown, because the two flagged bookings sit inside the period.</t>
+          <t>Step 9: The dialog closes. A green 'Unavailable period saved' message appears. Under 'Unavailable periods' a period is listed: 'Other', 'Film crew on site', 'Unavailable from 25 Jul 2027, 09:00. Available again from 26 Jul 2027, 09:00.'
+Step 12: The 25 Jul 2027 row lists 'Unavailable 09:00–24:00 · Other'. The 'Unavailable periods' card lists 'Other', 'Film crew on site', '25 Jul 2027, 09:00 – 26 Jul 2027, 09:00'.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4698,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46301</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">

</xml_diff>